<commit_message>
experiment 1 data collection and analysis
</commit_message>
<xml_diff>
--- a/Time to Fixation Experiments - Changing Chemotaxis Equation/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
+++ b/Time to Fixation Experiments - Changing Chemotaxis Equation/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Time to Fixation Experiments - Changing Chemotaxis Equation\Experiment 1 - Testing Fixation Time\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F35AFB-28CF-4026-A413-FD14DBD17ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E989EB-72A7-4461-8F64-9561082C1BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
   </bookViews>
@@ -1354,7 +1354,7 @@
         <v>1646</v>
       </c>
       <c r="D67">
-        <v>1757</v>
+        <v>9325</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -1634,7 +1634,7 @@
         <v>1358</v>
       </c>
       <c r="D87">
-        <v>1945</v>
+        <v>7096</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -1788,7 +1788,7 @@
         <v>1465</v>
       </c>
       <c r="D98">
-        <v>2414</v>
+        <v>7508</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -5238,9 +5238,11 @@
         <v>9325</v>
       </c>
       <c r="B2">
+        <f>A2/60</f>
         <v>155.41666666666666</v>
       </c>
       <c r="C2">
+        <f>A2/3600</f>
         <v>2.5902777777777777</v>
       </c>
     </row>
@@ -5249,9 +5251,11 @@
         <v>7508</v>
       </c>
       <c r="B3">
+        <f t="shared" ref="B3:B66" si="0">A3/60</f>
         <v>125.13333333333334</v>
       </c>
       <c r="C3">
+        <f t="shared" ref="C3:C66" si="1">A3/3600</f>
         <v>2.0855555555555556</v>
       </c>
     </row>
@@ -5260,9 +5264,11 @@
         <v>3453</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
         <v>57.55</v>
       </c>
       <c r="C4">
+        <f t="shared" si="1"/>
         <v>0.95916666666666661</v>
       </c>
     </row>
@@ -5271,9 +5277,11 @@
         <v>3480</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
         <v>58</v>
       </c>
       <c r="C5">
+        <f t="shared" si="1"/>
         <v>0.96666666666666667</v>
       </c>
     </row>
@@ -5282,9 +5290,11 @@
         <v>3649</v>
       </c>
       <c r="B6">
+        <f t="shared" si="0"/>
         <v>60.81666666666667</v>
       </c>
       <c r="C6">
+        <f t="shared" si="1"/>
         <v>1.013611111111111</v>
       </c>
     </row>
@@ -5293,9 +5303,11 @@
         <v>6902</v>
       </c>
       <c r="B7">
+        <f t="shared" si="0"/>
         <v>115.03333333333333</v>
       </c>
       <c r="C7">
+        <f t="shared" si="1"/>
         <v>1.9172222222222222</v>
       </c>
     </row>
@@ -5304,9 +5316,11 @@
         <v>4689</v>
       </c>
       <c r="B8">
+        <f t="shared" si="0"/>
         <v>78.150000000000006</v>
       </c>
       <c r="C8">
+        <f t="shared" si="1"/>
         <v>1.3025</v>
       </c>
     </row>
@@ -5315,9 +5329,11 @@
         <v>3570</v>
       </c>
       <c r="B9">
+        <f t="shared" si="0"/>
         <v>59.5</v>
       </c>
       <c r="C9">
+        <f t="shared" si="1"/>
         <v>0.9916666666666667</v>
       </c>
     </row>
@@ -5326,9 +5342,11 @@
         <v>4343</v>
       </c>
       <c r="B10">
+        <f t="shared" si="0"/>
         <v>72.38333333333334</v>
       </c>
       <c r="C10">
+        <f t="shared" si="1"/>
         <v>1.206388888888889</v>
       </c>
     </row>
@@ -5337,9 +5355,11 @@
         <v>7096</v>
       </c>
       <c r="B11">
+        <f t="shared" si="0"/>
         <v>118.26666666666667</v>
       </c>
       <c r="C11">
+        <f t="shared" si="1"/>
         <v>1.971111111111111</v>
       </c>
     </row>
@@ -5348,9 +5368,11 @@
         <v>4974</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
         <v>82.9</v>
       </c>
       <c r="C12">
+        <f t="shared" si="1"/>
         <v>1.3816666666666666</v>
       </c>
     </row>
@@ -5359,9 +5381,11 @@
         <v>6497</v>
       </c>
       <c r="B13">
+        <f t="shared" si="0"/>
         <v>108.28333333333333</v>
       </c>
       <c r="C13">
+        <f t="shared" si="1"/>
         <v>1.8047222222222221</v>
       </c>
     </row>
@@ -5370,9 +5394,11 @@
         <v>3064</v>
       </c>
       <c r="B14">
+        <f t="shared" si="0"/>
         <v>51.06666666666667</v>
       </c>
       <c r="C14">
+        <f t="shared" si="1"/>
         <v>0.85111111111111115</v>
       </c>
     </row>
@@ -5381,9 +5407,11 @@
         <v>3479</v>
       </c>
       <c r="B15">
+        <f t="shared" si="0"/>
         <v>57.983333333333334</v>
       </c>
       <c r="C15">
+        <f t="shared" si="1"/>
         <v>0.96638888888888885</v>
       </c>
     </row>
@@ -5392,9 +5420,11 @@
         <v>6799</v>
       </c>
       <c r="B16">
+        <f t="shared" si="0"/>
         <v>113.31666666666666</v>
       </c>
       <c r="C16">
+        <f t="shared" si="1"/>
         <v>1.888611111111111</v>
       </c>
     </row>
@@ -5403,9 +5433,11 @@
         <v>3771</v>
       </c>
       <c r="B17">
+        <f t="shared" si="0"/>
         <v>62.85</v>
       </c>
       <c r="C17">
+        <f t="shared" si="1"/>
         <v>1.0475000000000001</v>
       </c>
     </row>
@@ -5414,9 +5446,11 @@
         <v>5600</v>
       </c>
       <c r="B18">
+        <f t="shared" si="0"/>
         <v>93.333333333333329</v>
       </c>
       <c r="C18">
+        <f t="shared" si="1"/>
         <v>1.5555555555555556</v>
       </c>
     </row>
@@ -5425,9 +5459,11 @@
         <v>4370</v>
       </c>
       <c r="B19">
+        <f t="shared" si="0"/>
         <v>72.833333333333329</v>
       </c>
       <c r="C19">
+        <f t="shared" si="1"/>
         <v>1.2138888888888888</v>
       </c>
     </row>
@@ -5436,9 +5472,11 @@
         <v>4902</v>
       </c>
       <c r="B20">
+        <f t="shared" si="0"/>
         <v>81.7</v>
       </c>
       <c r="C20">
+        <f t="shared" si="1"/>
         <v>1.3616666666666666</v>
       </c>
     </row>
@@ -5447,9 +5485,11 @@
         <v>1974</v>
       </c>
       <c r="B21">
+        <f t="shared" si="0"/>
         <v>32.9</v>
       </c>
       <c r="C21">
+        <f t="shared" si="1"/>
         <v>0.54833333333333334</v>
       </c>
     </row>
@@ -5458,9 +5498,11 @@
         <v>4260</v>
       </c>
       <c r="B22">
+        <f t="shared" si="0"/>
         <v>71</v>
       </c>
       <c r="C22">
+        <f t="shared" si="1"/>
         <v>1.1833333333333333</v>
       </c>
     </row>
@@ -5469,9 +5511,11 @@
         <v>6671</v>
       </c>
       <c r="B23">
+        <f t="shared" si="0"/>
         <v>111.18333333333334</v>
       </c>
       <c r="C23">
+        <f t="shared" si="1"/>
         <v>1.8530555555555555</v>
       </c>
     </row>
@@ -5480,9 +5524,11 @@
         <v>5112</v>
       </c>
       <c r="B24">
+        <f t="shared" si="0"/>
         <v>85.2</v>
       </c>
       <c r="C24">
+        <f t="shared" si="1"/>
         <v>1.42</v>
       </c>
     </row>
@@ -5491,9 +5537,11 @@
         <v>4297</v>
       </c>
       <c r="B25">
+        <f t="shared" si="0"/>
         <v>71.61666666666666</v>
       </c>
       <c r="C25">
+        <f t="shared" si="1"/>
         <v>1.1936111111111112</v>
       </c>
     </row>
@@ -5502,9 +5550,11 @@
         <v>6984</v>
       </c>
       <c r="B26">
+        <f t="shared" si="0"/>
         <v>116.4</v>
       </c>
       <c r="C26">
+        <f t="shared" si="1"/>
         <v>1.94</v>
       </c>
     </row>
@@ -5513,9 +5563,11 @@
         <v>3434</v>
       </c>
       <c r="B27">
+        <f t="shared" si="0"/>
         <v>57.233333333333334</v>
       </c>
       <c r="C27">
+        <f t="shared" si="1"/>
         <v>0.9538888888888889</v>
       </c>
     </row>
@@ -5524,9 +5576,11 @@
         <v>9535</v>
       </c>
       <c r="B28">
+        <f t="shared" si="0"/>
         <v>158.91666666666666</v>
       </c>
       <c r="C28">
+        <f t="shared" si="1"/>
         <v>2.6486111111111112</v>
       </c>
     </row>
@@ -5535,9 +5589,11 @@
         <v>3505</v>
       </c>
       <c r="B29">
+        <f t="shared" si="0"/>
         <v>58.416666666666664</v>
       </c>
       <c r="C29">
+        <f t="shared" si="1"/>
         <v>0.97361111111111109</v>
       </c>
     </row>
@@ -5546,9 +5602,11 @@
         <v>6469</v>
       </c>
       <c r="B30">
+        <f t="shared" si="0"/>
         <v>107.81666666666666</v>
       </c>
       <c r="C30">
+        <f t="shared" si="1"/>
         <v>1.7969444444444445</v>
       </c>
     </row>
@@ -5557,9 +5615,11 @@
         <v>3314</v>
       </c>
       <c r="B31">
+        <f t="shared" si="0"/>
         <v>55.233333333333334</v>
       </c>
       <c r="C31">
+        <f t="shared" si="1"/>
         <v>0.92055555555555557</v>
       </c>
     </row>
@@ -5568,9 +5628,11 @@
         <v>5386</v>
       </c>
       <c r="B32">
+        <f t="shared" si="0"/>
         <v>89.766666666666666</v>
       </c>
       <c r="C32">
+        <f t="shared" si="1"/>
         <v>1.4961111111111112</v>
       </c>
     </row>
@@ -5579,9 +5641,11 @@
         <v>6845</v>
       </c>
       <c r="B33">
+        <f t="shared" si="0"/>
         <v>114.08333333333333</v>
       </c>
       <c r="C33">
+        <f t="shared" si="1"/>
         <v>1.9013888888888888</v>
       </c>
     </row>
@@ -5590,9 +5654,11 @@
         <v>5982</v>
       </c>
       <c r="B34">
+        <f t="shared" si="0"/>
         <v>99.7</v>
       </c>
       <c r="C34">
+        <f t="shared" si="1"/>
         <v>1.6616666666666666</v>
       </c>
     </row>
@@ -5601,9 +5667,11 @@
         <v>4212</v>
       </c>
       <c r="B35">
+        <f t="shared" si="0"/>
         <v>70.2</v>
       </c>
       <c r="C35">
+        <f t="shared" si="1"/>
         <v>1.17</v>
       </c>
     </row>
@@ -5612,9 +5680,11 @@
         <v>4286</v>
       </c>
       <c r="B36">
+        <f t="shared" si="0"/>
         <v>71.433333333333337</v>
       </c>
       <c r="C36">
+        <f t="shared" si="1"/>
         <v>1.1905555555555556</v>
       </c>
     </row>
@@ -5623,9 +5693,11 @@
         <v>8861</v>
       </c>
       <c r="B37">
+        <f t="shared" si="0"/>
         <v>147.68333333333334</v>
       </c>
       <c r="C37">
+        <f t="shared" si="1"/>
         <v>2.4613888888888891</v>
       </c>
     </row>
@@ -5634,9 +5706,11 @@
         <v>3815</v>
       </c>
       <c r="B38">
+        <f t="shared" si="0"/>
         <v>63.583333333333336</v>
       </c>
       <c r="C38">
+        <f t="shared" si="1"/>
         <v>1.0597222222222222</v>
       </c>
     </row>
@@ -5645,9 +5719,11 @@
         <v>2551</v>
       </c>
       <c r="B39">
+        <f t="shared" si="0"/>
         <v>42.516666666666666</v>
       </c>
       <c r="C39">
+        <f t="shared" si="1"/>
         <v>0.70861111111111108</v>
       </c>
     </row>
@@ -5656,9 +5732,11 @@
         <v>2960</v>
       </c>
       <c r="B40">
+        <f t="shared" si="0"/>
         <v>49.333333333333336</v>
       </c>
       <c r="C40">
+        <f t="shared" si="1"/>
         <v>0.82222222222222219</v>
       </c>
     </row>
@@ -5667,9 +5745,11 @@
         <v>8800</v>
       </c>
       <c r="B41">
+        <f t="shared" si="0"/>
         <v>146.66666666666666</v>
       </c>
       <c r="C41">
+        <f t="shared" si="1"/>
         <v>2.4444444444444446</v>
       </c>
     </row>
@@ -5678,9 +5758,11 @@
         <v>4259</v>
       </c>
       <c r="B42">
+        <f t="shared" si="0"/>
         <v>70.983333333333334</v>
       </c>
       <c r="C42">
+        <f t="shared" si="1"/>
         <v>1.1830555555555555</v>
       </c>
     </row>
@@ -5689,9 +5771,11 @@
         <v>5191</v>
       </c>
       <c r="B43">
+        <f t="shared" si="0"/>
         <v>86.516666666666666</v>
       </c>
       <c r="C43">
+        <f t="shared" si="1"/>
         <v>1.4419444444444445</v>
       </c>
     </row>
@@ -5700,9 +5784,11 @@
         <v>8252</v>
       </c>
       <c r="B44">
+        <f t="shared" si="0"/>
         <v>137.53333333333333</v>
       </c>
       <c r="C44">
+        <f t="shared" si="1"/>
         <v>2.2922222222222222</v>
       </c>
     </row>
@@ -5711,9 +5797,11 @@
         <v>9820</v>
       </c>
       <c r="B45">
+        <f t="shared" si="0"/>
         <v>163.66666666666666</v>
       </c>
       <c r="C45">
+        <f t="shared" si="1"/>
         <v>2.7277777777777779</v>
       </c>
     </row>
@@ -5722,9 +5810,11 @@
         <v>8256</v>
       </c>
       <c r="B46">
+        <f t="shared" si="0"/>
         <v>137.6</v>
       </c>
       <c r="C46">
+        <f t="shared" si="1"/>
         <v>2.2933333333333334</v>
       </c>
     </row>
@@ -5733,9 +5823,11 @@
         <v>7016</v>
       </c>
       <c r="B47">
+        <f t="shared" si="0"/>
         <v>116.93333333333334</v>
       </c>
       <c r="C47">
+        <f t="shared" si="1"/>
         <v>1.9488888888888889</v>
       </c>
     </row>
@@ -5744,9 +5836,11 @@
         <v>4037</v>
       </c>
       <c r="B48">
+        <f t="shared" si="0"/>
         <v>67.283333333333331</v>
       </c>
       <c r="C48">
+        <f t="shared" si="1"/>
         <v>1.121388888888889</v>
       </c>
     </row>
@@ -5755,9 +5849,11 @@
         <v>7135</v>
       </c>
       <c r="B49">
+        <f t="shared" si="0"/>
         <v>118.91666666666667</v>
       </c>
       <c r="C49">
+        <f t="shared" si="1"/>
         <v>1.9819444444444445</v>
       </c>
     </row>
@@ -5766,9 +5862,11 @@
         <v>4312</v>
       </c>
       <c r="B50">
+        <f t="shared" si="0"/>
         <v>71.86666666666666</v>
       </c>
       <c r="C50">
+        <f t="shared" si="1"/>
         <v>1.1977777777777778</v>
       </c>
     </row>
@@ -5777,9 +5875,11 @@
         <v>3613</v>
       </c>
       <c r="B51">
+        <f t="shared" si="0"/>
         <v>60.216666666666669</v>
       </c>
       <c r="C51">
+        <f t="shared" si="1"/>
         <v>1.003611111111111</v>
       </c>
     </row>
@@ -5788,9 +5888,11 @@
         <v>3792</v>
       </c>
       <c r="B52">
+        <f t="shared" si="0"/>
         <v>63.2</v>
       </c>
       <c r="C52">
+        <f t="shared" si="1"/>
         <v>1.0533333333333332</v>
       </c>
     </row>
@@ -5799,9 +5901,11 @@
         <v>3590</v>
       </c>
       <c r="B53">
+        <f t="shared" si="0"/>
         <v>59.833333333333336</v>
       </c>
       <c r="C53">
+        <f t="shared" si="1"/>
         <v>0.99722222222222223</v>
       </c>
     </row>
@@ -5810,9 +5914,11 @@
         <v>3048</v>
       </c>
       <c r="B54">
+        <f t="shared" si="0"/>
         <v>50.8</v>
       </c>
       <c r="C54">
+        <f t="shared" si="1"/>
         <v>0.84666666666666668</v>
       </c>
     </row>
@@ -5821,9 +5927,11 @@
         <v>3170</v>
       </c>
       <c r="B55">
+        <f t="shared" si="0"/>
         <v>52.833333333333336</v>
       </c>
       <c r="C55">
+        <f t="shared" si="1"/>
         <v>0.88055555555555554</v>
       </c>
     </row>
@@ -5832,9 +5940,11 @@
         <v>6534</v>
       </c>
       <c r="B56">
+        <f t="shared" si="0"/>
         <v>108.9</v>
       </c>
       <c r="C56">
+        <f t="shared" si="1"/>
         <v>1.8149999999999999</v>
       </c>
     </row>
@@ -5843,9 +5953,11 @@
         <v>2973</v>
       </c>
       <c r="B57">
+        <f t="shared" si="0"/>
         <v>49.55</v>
       </c>
       <c r="C57">
+        <f t="shared" si="1"/>
         <v>0.82583333333333331</v>
       </c>
     </row>
@@ -5854,9 +5966,11 @@
         <v>6903</v>
       </c>
       <c r="B58">
+        <f t="shared" si="0"/>
         <v>115.05</v>
       </c>
       <c r="C58">
+        <f t="shared" si="1"/>
         <v>1.9175</v>
       </c>
     </row>
@@ -5865,9 +5979,11 @@
         <v>6088</v>
       </c>
       <c r="B59">
+        <f t="shared" si="0"/>
         <v>101.46666666666667</v>
       </c>
       <c r="C59">
+        <f t="shared" si="1"/>
         <v>1.691111111111111</v>
       </c>
     </row>
@@ -5876,9 +5992,11 @@
         <v>5241</v>
       </c>
       <c r="B60">
+        <f t="shared" si="0"/>
         <v>87.35</v>
       </c>
       <c r="C60">
+        <f t="shared" si="1"/>
         <v>1.4558333333333333</v>
       </c>
     </row>
@@ -5887,9 +6005,11 @@
         <v>2337</v>
       </c>
       <c r="B61">
+        <f t="shared" si="0"/>
         <v>38.950000000000003</v>
       </c>
       <c r="C61">
+        <f t="shared" si="1"/>
         <v>0.64916666666666667</v>
       </c>
     </row>
@@ -5898,9 +6018,11 @@
         <v>5331</v>
       </c>
       <c r="B62">
+        <f t="shared" si="0"/>
         <v>88.85</v>
       </c>
       <c r="C62">
+        <f t="shared" si="1"/>
         <v>1.4808333333333332</v>
       </c>
     </row>
@@ -5909,9 +6031,11 @@
         <v>5944</v>
       </c>
       <c r="B63">
+        <f t="shared" si="0"/>
         <v>99.066666666666663</v>
       </c>
       <c r="C63">
+        <f t="shared" si="1"/>
         <v>1.6511111111111112</v>
       </c>
     </row>
@@ -5920,9 +6044,11 @@
         <v>4403</v>
       </c>
       <c r="B64">
+        <f t="shared" si="0"/>
         <v>73.38333333333334</v>
       </c>
       <c r="C64">
+        <f t="shared" si="1"/>
         <v>1.2230555555555556</v>
       </c>
     </row>
@@ -5931,9 +6057,11 @@
         <v>3123</v>
       </c>
       <c r="B65">
+        <f t="shared" si="0"/>
         <v>52.05</v>
       </c>
       <c r="C65">
+        <f t="shared" si="1"/>
         <v>0.86750000000000005</v>
       </c>
     </row>
@@ -5942,21 +6070,25 @@
         <v>4072</v>
       </c>
       <c r="B66">
+        <f t="shared" si="0"/>
         <v>67.86666666666666</v>
       </c>
       <c r="C66">
+        <f t="shared" si="1"/>
         <v>1.1311111111111112</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>1757</v>
+        <v>9325</v>
       </c>
       <c r="B67">
-        <v>29.283333333333335</v>
+        <f t="shared" ref="B67:B101" si="2">A67/60</f>
+        <v>155.41666666666666</v>
       </c>
       <c r="C67">
-        <v>0.48805555555555558</v>
+        <f t="shared" ref="C67:C101" si="3">A67/3600</f>
+        <v>2.5902777777777777</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -5964,9 +6096,11 @@
         <v>2771</v>
       </c>
       <c r="B68">
+        <f t="shared" si="2"/>
         <v>46.18333333333333</v>
       </c>
       <c r="C68">
+        <f t="shared" si="3"/>
         <v>0.7697222222222222</v>
       </c>
     </row>
@@ -5975,9 +6109,11 @@
         <v>3762</v>
       </c>
       <c r="B69">
+        <f t="shared" si="2"/>
         <v>62.7</v>
       </c>
       <c r="C69">
+        <f t="shared" si="3"/>
         <v>1.0449999999999999</v>
       </c>
     </row>
@@ -5986,9 +6122,11 @@
         <v>3108</v>
       </c>
       <c r="B70">
+        <f t="shared" si="2"/>
         <v>51.8</v>
       </c>
       <c r="C70">
+        <f t="shared" si="3"/>
         <v>0.86333333333333329</v>
       </c>
     </row>
@@ -5997,9 +6135,11 @@
         <v>3768</v>
       </c>
       <c r="B71">
+        <f t="shared" si="2"/>
         <v>62.8</v>
       </c>
       <c r="C71">
+        <f t="shared" si="3"/>
         <v>1.0466666666666666</v>
       </c>
     </row>
@@ -6008,9 +6148,11 @@
         <v>2954</v>
       </c>
       <c r="B72">
+        <f t="shared" si="2"/>
         <v>49.233333333333334</v>
       </c>
       <c r="C72">
+        <f t="shared" si="3"/>
         <v>0.82055555555555559</v>
       </c>
     </row>
@@ -6019,9 +6161,11 @@
         <v>6016</v>
       </c>
       <c r="B73">
+        <f t="shared" si="2"/>
         <v>100.26666666666667</v>
       </c>
       <c r="C73">
+        <f t="shared" si="3"/>
         <v>1.6711111111111112</v>
       </c>
     </row>
@@ -6030,9 +6174,11 @@
         <v>2642</v>
       </c>
       <c r="B74">
+        <f t="shared" si="2"/>
         <v>44.033333333333331</v>
       </c>
       <c r="C74">
+        <f t="shared" si="3"/>
         <v>0.73388888888888892</v>
       </c>
     </row>
@@ -6041,9 +6187,11 @@
         <v>5739</v>
       </c>
       <c r="B75">
+        <f t="shared" si="2"/>
         <v>95.65</v>
       </c>
       <c r="C75">
+        <f t="shared" si="3"/>
         <v>1.5941666666666667</v>
       </c>
     </row>
@@ -6052,9 +6200,11 @@
         <v>1982</v>
       </c>
       <c r="B76">
+        <f t="shared" si="2"/>
         <v>33.033333333333331</v>
       </c>
       <c r="C76">
+        <f t="shared" si="3"/>
         <v>0.55055555555555558</v>
       </c>
     </row>
@@ -6063,9 +6213,11 @@
         <v>3492</v>
       </c>
       <c r="B77">
+        <f t="shared" si="2"/>
         <v>58.2</v>
       </c>
       <c r="C77">
+        <f t="shared" si="3"/>
         <v>0.97</v>
       </c>
     </row>
@@ -6074,9 +6226,11 @@
         <v>3342</v>
       </c>
       <c r="B78">
+        <f t="shared" si="2"/>
         <v>55.7</v>
       </c>
       <c r="C78">
+        <f t="shared" si="3"/>
         <v>0.92833333333333334</v>
       </c>
     </row>
@@ -6085,9 +6239,11 @@
         <v>8504</v>
       </c>
       <c r="B79">
+        <f t="shared" si="2"/>
         <v>141.73333333333332</v>
       </c>
       <c r="C79">
+        <f t="shared" si="3"/>
         <v>2.362222222222222</v>
       </c>
     </row>
@@ -6096,9 +6252,11 @@
         <v>3413</v>
       </c>
       <c r="B80">
+        <f t="shared" si="2"/>
         <v>56.883333333333333</v>
       </c>
       <c r="C80">
+        <f t="shared" si="3"/>
         <v>0.94805555555555554</v>
       </c>
     </row>
@@ -6107,9 +6265,11 @@
         <v>5837</v>
       </c>
       <c r="B81">
+        <f t="shared" si="2"/>
         <v>97.283333333333331</v>
       </c>
       <c r="C81">
+        <f t="shared" si="3"/>
         <v>1.621388888888889</v>
       </c>
     </row>
@@ -6118,9 +6278,11 @@
         <v>6429</v>
       </c>
       <c r="B82">
+        <f t="shared" si="2"/>
         <v>107.15</v>
       </c>
       <c r="C82">
+        <f t="shared" si="3"/>
         <v>1.7858333333333334</v>
       </c>
     </row>
@@ -6129,9 +6291,11 @@
         <v>9512</v>
       </c>
       <c r="B83">
+        <f t="shared" si="2"/>
         <v>158.53333333333333</v>
       </c>
       <c r="C83">
+        <f t="shared" si="3"/>
         <v>2.6422222222222222</v>
       </c>
     </row>
@@ -6140,9 +6304,11 @@
         <v>5882</v>
       </c>
       <c r="B84">
+        <f t="shared" si="2"/>
         <v>98.033333333333331</v>
       </c>
       <c r="C84">
+        <f t="shared" si="3"/>
         <v>1.6338888888888889</v>
       </c>
     </row>
@@ -6151,9 +6317,11 @@
         <v>6908</v>
       </c>
       <c r="B85">
+        <f t="shared" si="2"/>
         <v>115.13333333333334</v>
       </c>
       <c r="C85">
+        <f t="shared" si="3"/>
         <v>1.9188888888888889</v>
       </c>
     </row>
@@ -6162,21 +6330,25 @@
         <v>7235</v>
       </c>
       <c r="B86">
+        <f t="shared" si="2"/>
         <v>120.58333333333333</v>
       </c>
       <c r="C86">
+        <f t="shared" si="3"/>
         <v>2.0097222222222224</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>1945</v>
+        <v>7096</v>
       </c>
       <c r="B87">
-        <v>32.416666666666664</v>
+        <f t="shared" si="2"/>
+        <v>118.26666666666667</v>
       </c>
       <c r="C87">
-        <v>0.54027777777777775</v>
+        <f t="shared" si="3"/>
+        <v>1.971111111111111</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -6184,9 +6356,11 @@
         <v>2387</v>
       </c>
       <c r="B88">
+        <f t="shared" si="2"/>
         <v>39.783333333333331</v>
       </c>
       <c r="C88">
+        <f t="shared" si="3"/>
         <v>0.66305555555555551</v>
       </c>
     </row>
@@ -6195,9 +6369,11 @@
         <v>8873</v>
       </c>
       <c r="B89">
+        <f t="shared" si="2"/>
         <v>147.88333333333333</v>
       </c>
       <c r="C89">
+        <f t="shared" si="3"/>
         <v>2.464722222222222</v>
       </c>
     </row>
@@ -6206,9 +6382,11 @@
         <v>7254</v>
       </c>
       <c r="B90">
+        <f t="shared" si="2"/>
         <v>120.9</v>
       </c>
       <c r="C90">
+        <f t="shared" si="3"/>
         <v>2.0150000000000001</v>
       </c>
     </row>
@@ -6217,9 +6395,11 @@
         <v>5294</v>
       </c>
       <c r="B91">
+        <f t="shared" si="2"/>
         <v>88.233333333333334</v>
       </c>
       <c r="C91">
+        <f t="shared" si="3"/>
         <v>1.4705555555555556</v>
       </c>
     </row>
@@ -6228,9 +6408,11 @@
         <v>2069</v>
       </c>
       <c r="B92">
+        <f t="shared" si="2"/>
         <v>34.483333333333334</v>
       </c>
       <c r="C92">
+        <f t="shared" si="3"/>
         <v>0.57472222222222225</v>
       </c>
     </row>
@@ -6239,9 +6421,11 @@
         <v>4272</v>
       </c>
       <c r="B93">
+        <f t="shared" si="2"/>
         <v>71.2</v>
       </c>
       <c r="C93">
+        <f t="shared" si="3"/>
         <v>1.1866666666666668</v>
       </c>
     </row>
@@ -6250,9 +6434,11 @@
         <v>7887</v>
       </c>
       <c r="B94">
+        <f t="shared" si="2"/>
         <v>131.44999999999999</v>
       </c>
       <c r="C94">
+        <f t="shared" si="3"/>
         <v>2.1908333333333334</v>
       </c>
     </row>
@@ -6261,9 +6447,11 @@
         <v>3106</v>
       </c>
       <c r="B95">
+        <f t="shared" si="2"/>
         <v>51.766666666666666</v>
       </c>
       <c r="C95">
+        <f t="shared" si="3"/>
         <v>0.86277777777777775</v>
       </c>
     </row>
@@ -6272,9 +6460,11 @@
         <v>6387</v>
       </c>
       <c r="B96">
+        <f t="shared" si="2"/>
         <v>106.45</v>
       </c>
       <c r="C96">
+        <f t="shared" si="3"/>
         <v>1.7741666666666667</v>
       </c>
     </row>
@@ -6283,21 +6473,25 @@
         <v>7081</v>
       </c>
       <c r="B97">
+        <f t="shared" si="2"/>
         <v>118.01666666666667</v>
       </c>
       <c r="C97">
+        <f t="shared" si="3"/>
         <v>1.9669444444444444</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>2414</v>
+        <v>7508</v>
       </c>
       <c r="B98">
-        <v>40.233333333333334</v>
+        <f t="shared" si="2"/>
+        <v>125.13333333333334</v>
       </c>
       <c r="C98">
-        <v>0.67055555555555557</v>
+        <f t="shared" si="3"/>
+        <v>2.0855555555555556</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -6305,9 +6499,11 @@
         <v>7013</v>
       </c>
       <c r="B99">
+        <f t="shared" si="2"/>
         <v>116.88333333333334</v>
       </c>
       <c r="C99">
+        <f t="shared" si="3"/>
         <v>1.9480555555555557</v>
       </c>
     </row>
@@ -6316,9 +6512,11 @@
         <v>4643</v>
       </c>
       <c r="B100">
+        <f t="shared" si="2"/>
         <v>77.38333333333334</v>
       </c>
       <c r="C100">
+        <f t="shared" si="3"/>
         <v>1.2897222222222222</v>
       </c>
     </row>
@@ -6327,9 +6525,11 @@
         <v>5652</v>
       </c>
       <c r="B101">
+        <f t="shared" si="2"/>
         <v>94.2</v>
       </c>
       <c r="C101">
+        <f t="shared" si="3"/>
         <v>1.57</v>
       </c>
     </row>

</xml_diff>